<commit_message>
work on dashboard for tuflow batch and log summary
</commit_message>
<xml_diff>
--- a/excel-tools/format_IFD.xlsx
+++ b/excel-tools/format_IFD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\BGER\PER\RP20180.317 WYLOO CREEK CROSSING PFS - FMG\4 ENGINEERING\11 HYDROLOGY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Library\Automation\ryan-tools\excel-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106404F6-B47E-4F57-BB42-507B59C0BC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23CBBBAD-8911-419A-912B-1B6C40D463EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{E1FEFACF-31CA-4DC4-BF45-269D09030C4E}"/>
+    <workbookView xWindow="-54600" yWindow="-2550" windowWidth="25800" windowHeight="21150" activeTab="1" xr2:uid="{E1FEFACF-31CA-4DC4-BF45-269D09030C4E}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_IFD" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="56">
   <si>
     <t>Copyright Commonwealth of Australia 2016 Bureau of Meteorology (ABN 92 637 533 532)</t>
   </si>
@@ -89,30 +89,6 @@
   </si>
   <si>
     <t>Duration</t>
-  </si>
-  <si>
-    <t>Duration in min</t>
-  </si>
-  <si>
-    <t>12EY</t>
-  </si>
-  <si>
-    <t>6EY</t>
-  </si>
-  <si>
-    <t>4EY</t>
-  </si>
-  <si>
-    <t>3EY</t>
-  </si>
-  <si>
-    <t>2EY</t>
-  </si>
-  <si>
-    <t>0.5EY</t>
-  </si>
-  <si>
-    <t>0.2EY</t>
   </si>
   <si>
     <t>1 in 200</t>
@@ -1128,20 +1104,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236D0590-E237-4CBD-8CA3-EB5706A6CD7F}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:T39"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1149,12 +1125,12 @@
         <v>45575</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1171,7 +1147,7 @@
         <v>117.00318</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -1179,16 +1155,16 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D7" t="s">
         <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>8</v>
       </c>
@@ -1196,1864 +1172,1237 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="D10" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="F10" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="H10" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="I10" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="J10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" t="s">
+      <c r="K10" t="s">
         <v>12</v>
       </c>
-      <c r="D10" t="s">
+      <c r="L10" t="s">
         <v>13</v>
       </c>
-      <c r="E10" t="s">
+      <c r="M10" t="s">
         <v>14</v>
       </c>
-      <c r="F10" t="s">
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>15</v>
-      </c>
-      <c r="G10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="6">
-        <v>0.63200000000000001</v>
-      </c>
-      <c r="I10" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="J10" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="L10" t="s">
-        <v>18</v>
-      </c>
-      <c r="M10" s="7">
-        <v>0.1</v>
-      </c>
-      <c r="N10" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="O10" s="7">
-        <v>0.02</v>
-      </c>
-      <c r="P10" s="7">
-        <v>0.01</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>19</v>
-      </c>
-      <c r="R10" t="s">
-        <v>20</v>
-      </c>
-      <c r="S10" t="s">
-        <v>21</v>
-      </c>
-      <c r="T10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>23</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11">
-        <v>0.42299999999999999</v>
+        <v>1.7</v>
       </c>
       <c r="D11">
-        <v>0.54800000000000004</v>
+        <v>1.97</v>
       </c>
       <c r="E11">
-        <v>0.77200000000000002</v>
+        <v>2.83</v>
       </c>
       <c r="F11">
-        <v>0.93799999999999994</v>
+        <v>3.42</v>
       </c>
       <c r="G11">
-        <v>1.18</v>
+        <v>4.01</v>
       </c>
       <c r="H11">
-        <v>1.63</v>
+        <v>4.79</v>
       </c>
       <c r="I11">
-        <v>1.88</v>
+        <v>5.39</v>
       </c>
       <c r="J11">
-        <v>2.09</v>
+        <v>6.14</v>
       </c>
       <c r="K11">
-        <v>2.68</v>
+        <v>7.25</v>
       </c>
       <c r="L11">
-        <v>2.73</v>
+        <v>8.14</v>
       </c>
       <c r="M11">
-        <v>3.22</v>
-      </c>
-      <c r="N11">
-        <v>3.76</v>
-      </c>
-      <c r="O11">
-        <v>4.4800000000000004</v>
-      </c>
-      <c r="P11">
-        <v>5.04</v>
-      </c>
-      <c r="Q11">
-        <v>5.77</v>
-      </c>
-      <c r="R11">
-        <v>6.88</v>
-      </c>
-      <c r="S11">
-        <v>7.79</v>
-      </c>
-      <c r="T11">
-        <v>8.76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12">
-        <v>0.73499999999999999</v>
+        <v>2.81</v>
       </c>
       <c r="D12">
-        <v>0.94799999999999995</v>
+        <v>3.25</v>
       </c>
       <c r="E12">
-        <v>1.32</v>
+        <v>4.6100000000000003</v>
       </c>
       <c r="F12">
-        <v>1.59</v>
+        <v>5.54</v>
       </c>
       <c r="G12">
-        <v>1.98</v>
+        <v>6.45</v>
       </c>
       <c r="H12">
-        <v>2.67</v>
+        <v>7.65</v>
       </c>
       <c r="I12">
-        <v>3.07</v>
+        <v>8.57</v>
       </c>
       <c r="J12">
-        <v>3.4</v>
+        <v>9.74</v>
       </c>
       <c r="K12">
-        <v>4.3</v>
+        <v>11.4</v>
       </c>
       <c r="L12">
-        <v>4.38</v>
+        <v>12.7</v>
       </c>
       <c r="M12">
-        <v>5.13</v>
-      </c>
-      <c r="N12">
-        <v>5.93</v>
-      </c>
-      <c r="O12">
-        <v>6.99</v>
-      </c>
-      <c r="P12">
-        <v>7.8</v>
-      </c>
-      <c r="Q12">
-        <v>9</v>
-      </c>
-      <c r="R12">
-        <v>10.8</v>
-      </c>
-      <c r="S12">
-        <v>12.2</v>
-      </c>
-      <c r="T12">
-        <v>13.7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B13">
         <v>3</v>
       </c>
       <c r="C13">
-        <v>1.03</v>
+        <v>3.97</v>
       </c>
       <c r="D13">
-        <v>1.33</v>
+        <v>4.59</v>
       </c>
       <c r="E13">
-        <v>1.87</v>
+        <v>6.55</v>
       </c>
       <c r="F13">
-        <v>2.25</v>
+        <v>7.88</v>
       </c>
       <c r="G13">
-        <v>2.8</v>
+        <v>9.19</v>
       </c>
       <c r="H13">
-        <v>3.77</v>
+        <v>10.9</v>
       </c>
       <c r="I13">
-        <v>4.33</v>
+        <v>12.3</v>
       </c>
       <c r="J13">
-        <v>4.8099999999999996</v>
+        <v>14</v>
       </c>
       <c r="K13">
-        <v>6.1</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="L13">
-        <v>6.22</v>
+        <v>18.3</v>
       </c>
       <c r="M13">
-        <v>7.3</v>
-      </c>
-      <c r="N13">
-        <v>8.4700000000000006</v>
-      </c>
-      <c r="O13">
-        <v>10</v>
-      </c>
-      <c r="P13">
-        <v>11.2</v>
-      </c>
-      <c r="Q13">
-        <v>12.9</v>
-      </c>
-      <c r="R13">
-        <v>15.4</v>
-      </c>
-      <c r="S13">
-        <v>17.399999999999999</v>
-      </c>
-      <c r="T13">
-        <v>19.600000000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+        <v>20.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>4</v>
       </c>
       <c r="C14">
-        <v>1.3</v>
+        <v>5.0599999999999996</v>
       </c>
       <c r="D14">
-        <v>1.69</v>
+        <v>5.86</v>
       </c>
       <c r="E14">
-        <v>2.37</v>
+        <v>8.39</v>
       </c>
       <c r="F14">
-        <v>2.87</v>
+        <v>10.1</v>
       </c>
       <c r="G14">
-        <v>3.57</v>
+        <v>11.8</v>
       </c>
       <c r="H14">
-        <v>4.8099999999999996</v>
+        <v>14.1</v>
       </c>
       <c r="I14">
-        <v>5.54</v>
+        <v>15.9</v>
       </c>
       <c r="J14">
-        <v>6.15</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="K14">
-        <v>7.84</v>
+        <v>21.2</v>
       </c>
       <c r="L14">
-        <v>7.99</v>
+        <v>23.8</v>
       </c>
       <c r="M14">
-        <v>9.4</v>
-      </c>
-      <c r="N14">
-        <v>10.9</v>
-      </c>
-      <c r="O14">
-        <v>13</v>
-      </c>
-      <c r="P14">
-        <v>14.5</v>
-      </c>
-      <c r="Q14">
-        <v>16.7</v>
-      </c>
-      <c r="R14">
-        <v>19.899999999999999</v>
-      </c>
-      <c r="S14">
-        <v>22.5</v>
-      </c>
-      <c r="T14">
-        <v>25.4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+        <v>26.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B15">
         <v>5</v>
       </c>
       <c r="C15">
-        <v>1.55</v>
+        <v>6.07</v>
       </c>
       <c r="D15">
-        <v>2.02</v>
+        <v>7.04</v>
       </c>
       <c r="E15">
-        <v>2.84</v>
+        <v>10.1</v>
       </c>
       <c r="F15">
-        <v>3.43</v>
+        <v>12.2</v>
       </c>
       <c r="G15">
-        <v>4.28</v>
+        <v>14.3</v>
       </c>
       <c r="H15">
-        <v>5.77</v>
+        <v>17</v>
       </c>
       <c r="I15">
-        <v>6.66</v>
+        <v>19.2</v>
       </c>
       <c r="J15">
-        <v>7.39</v>
+        <v>21.9</v>
       </c>
       <c r="K15">
-        <v>9.4499999999999993</v>
+        <v>25.7</v>
       </c>
       <c r="L15">
-        <v>9.64</v>
+        <v>28.9</v>
       </c>
       <c r="M15">
-        <v>11.4</v>
-      </c>
-      <c r="N15">
-        <v>13.2</v>
-      </c>
-      <c r="O15">
-        <v>15.7</v>
-      </c>
-      <c r="P15">
-        <v>17.7</v>
-      </c>
-      <c r="Q15">
-        <v>20.3</v>
-      </c>
-      <c r="R15">
-        <v>24.2</v>
-      </c>
-      <c r="S15">
-        <v>27.3</v>
-      </c>
-      <c r="T15">
-        <v>30.8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+        <v>32.200000000000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B16">
         <v>10</v>
       </c>
       <c r="C16">
-        <v>2.5099999999999998</v>
+        <v>10.1</v>
       </c>
       <c r="D16">
-        <v>3.29</v>
+        <v>11.7</v>
       </c>
       <c r="E16">
-        <v>4.66</v>
+        <v>16.8</v>
       </c>
       <c r="F16">
-        <v>5.66</v>
+        <v>20.3</v>
       </c>
       <c r="G16">
-        <v>7.09</v>
+        <v>23.8</v>
       </c>
       <c r="H16">
-        <v>9.6</v>
+        <v>28.5</v>
       </c>
       <c r="I16">
-        <v>11.1</v>
+        <v>32.1</v>
       </c>
       <c r="J16">
-        <v>12.3</v>
+        <v>36.6</v>
       </c>
       <c r="K16">
-        <v>15.8</v>
+        <v>43.3</v>
       </c>
       <c r="L16">
-        <v>16.100000000000001</v>
+        <v>48.7</v>
       </c>
       <c r="M16">
-        <v>19.100000000000001</v>
-      </c>
-      <c r="N16">
-        <v>22.3</v>
-      </c>
-      <c r="O16">
-        <v>26.6</v>
-      </c>
-      <c r="P16">
-        <v>30</v>
-      </c>
-      <c r="Q16">
-        <v>34.299999999999997</v>
-      </c>
-      <c r="R16">
-        <v>40.799999999999997</v>
-      </c>
-      <c r="S16">
-        <v>46.2</v>
-      </c>
-      <c r="T16">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B17">
         <v>15</v>
       </c>
       <c r="C17">
-        <v>3.18</v>
+        <v>12.8</v>
       </c>
       <c r="D17">
-        <v>4.17</v>
+        <v>14.9</v>
       </c>
       <c r="E17">
-        <v>5.93</v>
+        <v>21.4</v>
       </c>
       <c r="F17">
-        <v>7.2</v>
+        <v>25.9</v>
       </c>
       <c r="G17">
-        <v>9.0399999999999991</v>
+        <v>30.3</v>
       </c>
       <c r="H17">
-        <v>12.3</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="I17">
-        <v>14.2</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="J17">
-        <v>15.7</v>
+        <v>46.5</v>
       </c>
       <c r="K17">
-        <v>20.2</v>
+        <v>55</v>
       </c>
       <c r="L17">
-        <v>20.6</v>
+        <v>61.8</v>
       </c>
       <c r="M17">
-        <v>24.4</v>
-      </c>
-      <c r="N17">
-        <v>28.5</v>
-      </c>
-      <c r="O17">
-        <v>34</v>
-      </c>
-      <c r="P17">
-        <v>38.299999999999997</v>
-      </c>
-      <c r="Q17">
-        <v>43.8</v>
-      </c>
-      <c r="R17">
-        <v>52.2</v>
-      </c>
-      <c r="S17">
-        <v>59.1</v>
-      </c>
-      <c r="T17">
-        <v>66.400000000000006</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+        <v>69.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B18">
         <v>20</v>
       </c>
       <c r="C18">
-        <v>3.68</v>
+        <v>14.9</v>
       </c>
       <c r="D18">
-        <v>4.84</v>
+        <v>17.3</v>
       </c>
       <c r="E18">
-        <v>6.88</v>
+        <v>24.8</v>
       </c>
       <c r="F18">
-        <v>8.36</v>
+        <v>30</v>
       </c>
       <c r="G18">
-        <v>10.5</v>
+        <v>35.1</v>
       </c>
       <c r="H18">
-        <v>14.3</v>
+        <v>41.9</v>
       </c>
       <c r="I18">
-        <v>16.5</v>
+        <v>47.1</v>
       </c>
       <c r="J18">
-        <v>18.3</v>
+        <v>53.7</v>
       </c>
       <c r="K18">
-        <v>23.5</v>
+        <v>63.5</v>
       </c>
       <c r="L18">
-        <v>24</v>
+        <v>71.3</v>
       </c>
       <c r="M18">
-        <v>28.3</v>
-      </c>
-      <c r="N18">
-        <v>33.1</v>
-      </c>
-      <c r="O18">
-        <v>39.4</v>
-      </c>
-      <c r="P18">
-        <v>44.3</v>
-      </c>
-      <c r="Q18">
-        <v>50.8</v>
-      </c>
-      <c r="R18">
-        <v>60.5</v>
-      </c>
-      <c r="S18">
-        <v>68.5</v>
-      </c>
-      <c r="T18">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+        <v>79.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B19">
         <v>25</v>
       </c>
       <c r="C19">
-        <v>4.08</v>
+        <v>16.5</v>
       </c>
       <c r="D19">
-        <v>5.36</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="E19">
-        <v>7.62</v>
+        <v>27.5</v>
       </c>
       <c r="F19">
-        <v>9.26</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="G19">
-        <v>11.6</v>
+        <v>38.799999999999997</v>
       </c>
       <c r="H19">
-        <v>15.9</v>
+        <v>46.3</v>
       </c>
       <c r="I19">
-        <v>18.3</v>
+        <v>52.1</v>
       </c>
       <c r="J19">
-        <v>20.3</v>
+        <v>59.4</v>
       </c>
       <c r="K19">
-        <v>26.1</v>
+        <v>70.099999999999994</v>
       </c>
       <c r="L19">
-        <v>26.6</v>
+        <v>78.7</v>
       </c>
       <c r="M19">
-        <v>31.4</v>
-      </c>
-      <c r="N19">
-        <v>36.6</v>
-      </c>
-      <c r="O19">
-        <v>43.6</v>
-      </c>
-      <c r="P19">
-        <v>49</v>
-      </c>
-      <c r="Q19">
-        <v>56.2</v>
-      </c>
-      <c r="R19">
-        <v>66.900000000000006</v>
-      </c>
-      <c r="S19">
-        <v>75.8</v>
-      </c>
-      <c r="T19">
-        <v>85.3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B20">
         <v>30</v>
       </c>
       <c r="C20">
-        <v>4.4000000000000004</v>
+        <v>17.8</v>
       </c>
       <c r="D20">
-        <v>5.79</v>
+        <v>20.7</v>
       </c>
       <c r="E20">
-        <v>8.23</v>
+        <v>29.6</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="G20">
-        <v>12.6</v>
+        <v>41.8</v>
       </c>
       <c r="H20">
-        <v>17.2</v>
+        <v>49.9</v>
       </c>
       <c r="I20">
-        <v>19.8</v>
+        <v>56.1</v>
       </c>
       <c r="J20">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="K20">
-        <v>28.2</v>
+        <v>75.5</v>
       </c>
       <c r="L20">
-        <v>28.7</v>
+        <v>84.7</v>
       </c>
       <c r="M20">
-        <v>33.9</v>
-      </c>
-      <c r="N20">
-        <v>39.5</v>
-      </c>
-      <c r="O20">
-        <v>47</v>
-      </c>
-      <c r="P20">
-        <v>52.8</v>
-      </c>
-      <c r="Q20">
-        <v>60.6</v>
-      </c>
-      <c r="R20">
-        <v>72.2</v>
-      </c>
-      <c r="S20">
-        <v>81.7</v>
-      </c>
-      <c r="T20">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+        <v>94.6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B21">
         <v>45</v>
       </c>
       <c r="C21">
-        <v>5.1100000000000003</v>
+        <v>20.7</v>
       </c>
       <c r="D21">
-        <v>6.72</v>
+        <v>24</v>
       </c>
       <c r="E21">
-        <v>9.56</v>
+        <v>34.5</v>
       </c>
       <c r="F21">
-        <v>11.6</v>
+        <v>41.6</v>
       </c>
       <c r="G21">
-        <v>14.6</v>
+        <v>48.7</v>
       </c>
       <c r="H21">
-        <v>20.100000000000001</v>
+        <v>58.1</v>
       </c>
       <c r="I21">
-        <v>23.2</v>
+        <v>65.3</v>
       </c>
       <c r="J21">
-        <v>25.7</v>
+        <v>74.400000000000006</v>
       </c>
       <c r="K21">
-        <v>32.799999999999997</v>
+        <v>87.7</v>
       </c>
       <c r="L21">
-        <v>33.5</v>
+        <v>98.4</v>
       </c>
       <c r="M21">
-        <v>39.4</v>
-      </c>
-      <c r="N21">
-        <v>46</v>
-      </c>
-      <c r="O21">
-        <v>54.6</v>
-      </c>
-      <c r="P21">
-        <v>61.3</v>
-      </c>
-      <c r="Q21">
-        <v>70.400000000000006</v>
-      </c>
-      <c r="R21">
-        <v>83.9</v>
-      </c>
-      <c r="S21">
-        <v>95</v>
-      </c>
-      <c r="T21">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B22">
         <v>60</v>
       </c>
       <c r="C22">
-        <v>5.58</v>
+        <v>22.8</v>
       </c>
       <c r="D22">
-        <v>7.35</v>
+        <v>26.4</v>
       </c>
       <c r="E22">
-        <v>10.5</v>
+        <v>37.9</v>
       </c>
       <c r="F22">
-        <v>12.8</v>
+        <v>45.8</v>
       </c>
       <c r="G22">
-        <v>16.100000000000001</v>
+        <v>53.7</v>
       </c>
       <c r="H22">
-        <v>22.1</v>
+        <v>64.099999999999994</v>
       </c>
       <c r="I22">
-        <v>25.5</v>
+        <v>72.2</v>
       </c>
       <c r="J22">
-        <v>28.3</v>
+        <v>82.3</v>
       </c>
       <c r="K22">
-        <v>36.200000000000003</v>
+        <v>96.8</v>
       </c>
       <c r="L22">
-        <v>36.9</v>
+        <v>109</v>
       </c>
       <c r="M22">
-        <v>43.4</v>
-      </c>
-      <c r="N22">
-        <v>50.6</v>
-      </c>
-      <c r="O22">
-        <v>60.2</v>
-      </c>
-      <c r="P22">
-        <v>67.599999999999994</v>
-      </c>
-      <c r="Q22">
-        <v>77.5</v>
-      </c>
-      <c r="R22">
-        <v>92.5</v>
-      </c>
-      <c r="S22">
-        <v>105</v>
-      </c>
-      <c r="T22">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B23">
         <v>90</v>
       </c>
       <c r="C23">
-        <v>6.2</v>
+        <v>25.7</v>
       </c>
       <c r="D23">
-        <v>8.18</v>
+        <v>29.8</v>
       </c>
       <c r="E23">
-        <v>11.7</v>
+        <v>43</v>
       </c>
       <c r="F23">
-        <v>14.3</v>
+        <v>52.1</v>
       </c>
       <c r="G23">
-        <v>18.100000000000001</v>
+        <v>61.2</v>
       </c>
       <c r="H23">
-        <v>25</v>
+        <v>73.400000000000006</v>
       </c>
       <c r="I23">
-        <v>28.8</v>
+        <v>83</v>
       </c>
       <c r="J23">
-        <v>32</v>
+        <v>94.5</v>
       </c>
       <c r="K23">
-        <v>41</v>
+        <v>111</v>
       </c>
       <c r="L23">
-        <v>41.8</v>
+        <v>125</v>
       </c>
       <c r="M23">
-        <v>49.3</v>
-      </c>
-      <c r="N23">
-        <v>57.5</v>
-      </c>
-      <c r="O23">
-        <v>68.5</v>
-      </c>
-      <c r="P23">
-        <v>77</v>
-      </c>
-      <c r="Q23">
-        <v>88.4</v>
-      </c>
-      <c r="R23">
-        <v>105</v>
-      </c>
-      <c r="S23">
-        <v>119</v>
-      </c>
-      <c r="T23">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B24">
         <v>120</v>
       </c>
       <c r="C24">
-        <v>6.61</v>
+        <v>27.8</v>
       </c>
       <c r="D24">
-        <v>8.75</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="E24">
-        <v>12.6</v>
+        <v>46.9</v>
       </c>
       <c r="F24">
-        <v>15.4</v>
+        <v>57.1</v>
       </c>
       <c r="G24">
-        <v>19.5</v>
+        <v>67.2</v>
       </c>
       <c r="H24">
-        <v>27.1</v>
+        <v>80.900000000000006</v>
       </c>
       <c r="I24">
-        <v>31.3</v>
+        <v>91.7</v>
       </c>
       <c r="J24">
-        <v>34.700000000000003</v>
+        <v>104</v>
       </c>
       <c r="K24">
-        <v>44.6</v>
+        <v>123</v>
       </c>
       <c r="L24">
-        <v>45.5</v>
+        <v>138</v>
       </c>
       <c r="M24">
-        <v>53.8</v>
-      </c>
-      <c r="N24">
-        <v>62.9</v>
-      </c>
-      <c r="O24">
-        <v>75.099999999999994</v>
-      </c>
-      <c r="P24">
-        <v>84.6</v>
-      </c>
-      <c r="Q24">
-        <v>97</v>
-      </c>
-      <c r="R24">
-        <v>116</v>
-      </c>
-      <c r="S24">
-        <v>131</v>
-      </c>
-      <c r="T24">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B25">
         <v>180</v>
       </c>
       <c r="C25">
-        <v>7.15</v>
+        <v>31</v>
       </c>
       <c r="D25">
-        <v>9.5</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="E25">
-        <v>13.7</v>
+        <v>53</v>
       </c>
       <c r="F25">
-        <v>16.899999999999999</v>
+        <v>64.900000000000006</v>
       </c>
       <c r="G25">
-        <v>21.5</v>
+        <v>76.900000000000006</v>
       </c>
       <c r="H25">
+        <v>93.4</v>
+      </c>
+      <c r="I25">
+        <v>106</v>
+      </c>
+      <c r="J25">
+        <v>121</v>
+      </c>
+      <c r="K25">
+        <v>143</v>
+      </c>
+      <c r="L25">
+        <v>160</v>
+      </c>
+      <c r="M25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>30</v>
-      </c>
-      <c r="I25">
-        <v>34.799999999999997</v>
-      </c>
-      <c r="J25">
-        <v>38.700000000000003</v>
-      </c>
-      <c r="K25">
-        <v>50.2</v>
-      </c>
-      <c r="L25">
-        <v>51.2</v>
-      </c>
-      <c r="M25">
-        <v>60.9</v>
-      </c>
-      <c r="N25">
-        <v>71.5</v>
-      </c>
-      <c r="O25">
-        <v>85.9</v>
-      </c>
-      <c r="P25">
-        <v>97.2</v>
-      </c>
-      <c r="Q25">
-        <v>111</v>
-      </c>
-      <c r="R25">
-        <v>133</v>
-      </c>
-      <c r="S25">
-        <v>150</v>
-      </c>
-      <c r="T25">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>38</v>
       </c>
       <c r="B26">
         <v>270</v>
       </c>
       <c r="C26">
-        <v>7.67</v>
+        <v>34.5</v>
       </c>
       <c r="D26">
-        <v>10.199999999999999</v>
+        <v>40.6</v>
       </c>
       <c r="E26">
-        <v>14.9</v>
+        <v>60.3</v>
       </c>
       <c r="F26">
-        <v>18.399999999999999</v>
+        <v>74.400000000000006</v>
       </c>
       <c r="G26">
-        <v>23.6</v>
+        <v>88.7</v>
       </c>
       <c r="H26">
-        <v>33.1</v>
+        <v>109</v>
       </c>
       <c r="I26">
-        <v>38.700000000000003</v>
+        <v>125</v>
       </c>
       <c r="J26">
-        <v>42.9</v>
+        <v>142</v>
       </c>
       <c r="K26">
-        <v>56.5</v>
+        <v>168</v>
       </c>
       <c r="L26">
-        <v>57.6</v>
+        <v>189</v>
       </c>
       <c r="M26">
-        <v>69</v>
-      </c>
-      <c r="N26">
-        <v>81.599999999999994</v>
-      </c>
-      <c r="O26">
-        <v>98.9</v>
-      </c>
-      <c r="P26">
-        <v>113</v>
-      </c>
-      <c r="Q26">
-        <v>129</v>
-      </c>
-      <c r="R26">
-        <v>153</v>
-      </c>
-      <c r="S26">
-        <v>173</v>
-      </c>
-      <c r="T26">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B27">
         <v>360</v>
       </c>
       <c r="C27">
-        <v>8.0299999999999994</v>
+        <v>37.4</v>
       </c>
       <c r="D27">
-        <v>10.8</v>
+        <v>44.1</v>
       </c>
       <c r="E27">
-        <v>15.8</v>
+        <v>66.2</v>
       </c>
       <c r="F27">
-        <v>19.5</v>
+        <v>82.2</v>
       </c>
       <c r="G27">
-        <v>25.1</v>
+        <v>98.7</v>
       </c>
       <c r="H27">
-        <v>35.5</v>
+        <v>122</v>
       </c>
       <c r="I27">
-        <v>41.6</v>
+        <v>140</v>
       </c>
       <c r="J27">
-        <v>46.1</v>
+        <v>160</v>
       </c>
       <c r="K27">
-        <v>61.4</v>
+        <v>189</v>
       </c>
       <c r="L27">
-        <v>62.6</v>
+        <v>213</v>
       </c>
       <c r="M27">
-        <v>75.5</v>
-      </c>
-      <c r="N27">
-        <v>89.9</v>
-      </c>
-      <c r="O27">
-        <v>110</v>
-      </c>
-      <c r="P27">
-        <v>125</v>
-      </c>
-      <c r="Q27">
-        <v>143</v>
-      </c>
-      <c r="R27">
-        <v>171</v>
-      </c>
-      <c r="S27">
-        <v>193</v>
-      </c>
-      <c r="T27">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B28">
         <v>540</v>
       </c>
       <c r="C28">
-        <v>8.5399999999999991</v>
+        <v>42</v>
       </c>
       <c r="D28">
-        <v>11.5</v>
+        <v>49.8</v>
       </c>
       <c r="E28">
-        <v>17</v>
+        <v>76</v>
       </c>
       <c r="F28">
-        <v>21.1</v>
+        <v>95.2</v>
       </c>
       <c r="G28">
-        <v>27.3</v>
+        <v>115</v>
       </c>
       <c r="H28">
-        <v>38.9</v>
+        <v>143</v>
       </c>
       <c r="I28">
-        <v>45.9</v>
+        <v>166</v>
       </c>
       <c r="J28">
-        <v>50.9</v>
+        <v>189</v>
       </c>
       <c r="K28">
-        <v>69</v>
+        <v>224</v>
       </c>
       <c r="L28">
-        <v>70.400000000000006</v>
+        <v>252</v>
       </c>
       <c r="M28">
-        <v>85.8</v>
-      </c>
-      <c r="N28">
-        <v>103</v>
-      </c>
-      <c r="O28">
-        <v>127</v>
-      </c>
-      <c r="P28">
-        <v>147</v>
-      </c>
-      <c r="Q28">
-        <v>167</v>
-      </c>
-      <c r="R28">
-        <v>199</v>
-      </c>
-      <c r="S28">
-        <v>225</v>
-      </c>
-      <c r="T28">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B29">
         <v>720</v>
       </c>
       <c r="C29">
-        <v>8.92</v>
+        <v>45.7</v>
       </c>
       <c r="D29">
-        <v>12.1</v>
+        <v>54.4</v>
       </c>
       <c r="E29">
-        <v>17.899999999999999</v>
+        <v>83.9</v>
       </c>
       <c r="F29">
-        <v>22.3</v>
+        <v>106</v>
       </c>
       <c r="G29">
-        <v>28.9</v>
+        <v>128</v>
       </c>
       <c r="H29">
-        <v>41.5</v>
+        <v>160</v>
       </c>
       <c r="I29">
-        <v>49.1</v>
+        <v>186</v>
       </c>
       <c r="J29">
-        <v>54.5</v>
+        <v>213</v>
       </c>
       <c r="K29">
-        <v>74.8</v>
+        <v>252</v>
       </c>
       <c r="L29">
-        <v>76.3</v>
+        <v>284</v>
       </c>
       <c r="M29">
-        <v>93.7</v>
-      </c>
-      <c r="N29">
-        <v>113</v>
-      </c>
-      <c r="O29">
-        <v>141</v>
-      </c>
-      <c r="P29">
-        <v>164</v>
-      </c>
-      <c r="Q29">
-        <v>187</v>
-      </c>
-      <c r="R29">
-        <v>222</v>
-      </c>
-      <c r="S29">
-        <v>251</v>
-      </c>
-      <c r="T29">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>1080</v>
       </c>
       <c r="C30">
-        <v>9.49</v>
+        <v>51.5</v>
       </c>
       <c r="D30">
-        <v>12.9</v>
+        <v>61.7</v>
       </c>
       <c r="E30">
-        <v>19.2</v>
+        <v>96.4</v>
       </c>
       <c r="F30">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="G30">
-        <v>31.2</v>
+        <v>149</v>
       </c>
       <c r="H30">
-        <v>45.1</v>
+        <v>187</v>
       </c>
       <c r="I30">
-        <v>53.8</v>
+        <v>218</v>
       </c>
       <c r="J30">
-        <v>59.7</v>
+        <v>248</v>
       </c>
       <c r="K30">
-        <v>83.2</v>
+        <v>293</v>
       </c>
       <c r="L30">
-        <v>84.9</v>
+        <v>330</v>
       </c>
       <c r="M30">
-        <v>105</v>
-      </c>
-      <c r="N30">
-        <v>129</v>
-      </c>
-      <c r="O30">
-        <v>162</v>
-      </c>
-      <c r="P30">
-        <v>189</v>
-      </c>
-      <c r="Q30">
-        <v>216</v>
-      </c>
-      <c r="R30">
-        <v>257</v>
-      </c>
-      <c r="S30">
-        <v>291</v>
-      </c>
-      <c r="T30">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B31">
         <v>1440</v>
       </c>
       <c r="C31">
-        <v>9.91</v>
+        <v>56</v>
       </c>
       <c r="D31">
-        <v>13.5</v>
+        <v>67.400000000000006</v>
       </c>
       <c r="E31">
-        <v>20.100000000000001</v>
+        <v>106</v>
       </c>
       <c r="F31">
-        <v>25.2</v>
+        <v>135</v>
       </c>
       <c r="G31">
-        <v>32.9</v>
+        <v>165</v>
       </c>
       <c r="H31">
-        <v>47.7</v>
+        <v>206</v>
       </c>
       <c r="I31">
-        <v>57</v>
+        <v>240</v>
       </c>
       <c r="J31">
-        <v>63.3</v>
+        <v>274</v>
       </c>
       <c r="K31">
-        <v>89.2</v>
+        <v>323</v>
       </c>
       <c r="L31">
-        <v>91</v>
+        <v>362</v>
       </c>
       <c r="M31">
-        <v>114</v>
-      </c>
-      <c r="N31">
-        <v>140</v>
-      </c>
-      <c r="O31">
-        <v>176</v>
-      </c>
-      <c r="P31">
-        <v>207</v>
-      </c>
-      <c r="Q31">
-        <v>237</v>
-      </c>
-      <c r="R31">
-        <v>282</v>
-      </c>
-      <c r="S31">
-        <v>320</v>
-      </c>
-      <c r="T31">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B32">
         <v>1800</v>
       </c>
       <c r="C32">
-        <v>10.199999999999999</v>
+        <v>59.7</v>
       </c>
       <c r="D32">
-        <v>14</v>
+        <v>72</v>
       </c>
       <c r="E32">
-        <v>20.8</v>
+        <v>114</v>
       </c>
       <c r="F32">
-        <v>26.1</v>
+        <v>144</v>
       </c>
       <c r="G32">
-        <v>34.1</v>
+        <v>177</v>
       </c>
       <c r="H32">
-        <v>49.6</v>
+        <v>221</v>
       </c>
       <c r="I32">
-        <v>59.5</v>
+        <v>257</v>
       </c>
       <c r="J32">
-        <v>66.099999999999994</v>
+        <v>294</v>
       </c>
       <c r="K32">
-        <v>93.7</v>
+        <v>347</v>
       </c>
       <c r="L32">
-        <v>95.5</v>
+        <v>390</v>
       </c>
       <c r="M32">
-        <v>120</v>
-      </c>
-      <c r="N32">
-        <v>148</v>
-      </c>
-      <c r="O32">
-        <v>187</v>
-      </c>
-      <c r="P32">
-        <v>220</v>
-      </c>
-      <c r="Q32">
-        <v>256</v>
-      </c>
-      <c r="R32">
-        <v>305</v>
-      </c>
-      <c r="S32">
-        <v>346</v>
-      </c>
-      <c r="T32">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B33">
         <v>2160</v>
       </c>
       <c r="C33">
-        <v>10.5</v>
+        <v>62.7</v>
       </c>
       <c r="D33">
-        <v>14.4</v>
+        <v>75.8</v>
       </c>
       <c r="E33">
-        <v>21.4</v>
+        <v>120</v>
       </c>
       <c r="F33">
-        <v>26.8</v>
+        <v>152</v>
       </c>
       <c r="G33">
-        <v>35.1</v>
+        <v>186</v>
       </c>
       <c r="H33">
-        <v>51.2</v>
+        <v>232</v>
       </c>
       <c r="I33">
-        <v>61.5</v>
+        <v>269</v>
       </c>
       <c r="J33">
-        <v>68.3</v>
+        <v>308</v>
       </c>
       <c r="K33">
-        <v>97.2</v>
+        <v>363</v>
       </c>
       <c r="L33">
-        <v>99.1</v>
+        <v>407</v>
       </c>
       <c r="M33">
-        <v>124</v>
-      </c>
-      <c r="N33">
-        <v>154</v>
-      </c>
-      <c r="O33">
-        <v>195</v>
-      </c>
-      <c r="P33">
-        <v>230</v>
-      </c>
-      <c r="Q33">
-        <v>268</v>
-      </c>
-      <c r="R33">
-        <v>320</v>
-      </c>
-      <c r="S33">
-        <v>364</v>
-      </c>
-      <c r="T33">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B34">
         <v>2880</v>
       </c>
       <c r="C34">
-        <v>10.9</v>
+        <v>67.599999999999994</v>
       </c>
       <c r="D34">
-        <v>14.9</v>
+        <v>81.7</v>
       </c>
       <c r="E34">
-        <v>22.3</v>
+        <v>129</v>
       </c>
       <c r="F34">
-        <v>28</v>
+        <v>164</v>
       </c>
       <c r="G34">
-        <v>36.6</v>
+        <v>200</v>
       </c>
       <c r="H34">
-        <v>53.7</v>
+        <v>248</v>
       </c>
       <c r="I34">
-        <v>64.5</v>
+        <v>286</v>
       </c>
       <c r="J34">
-        <v>71.599999999999994</v>
+        <v>326</v>
       </c>
       <c r="K34">
-        <v>102</v>
+        <v>381</v>
       </c>
       <c r="L34">
-        <v>104</v>
+        <v>425</v>
       </c>
       <c r="M34">
-        <v>131</v>
-      </c>
-      <c r="N34">
-        <v>163</v>
-      </c>
-      <c r="O34">
-        <v>207</v>
-      </c>
-      <c r="P34">
-        <v>243</v>
-      </c>
-      <c r="Q34">
-        <v>284</v>
-      </c>
-      <c r="R34">
-        <v>339</v>
-      </c>
-      <c r="S34">
-        <v>386</v>
-      </c>
-      <c r="T34">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B35">
         <v>4320</v>
       </c>
       <c r="C35">
-        <v>11.5</v>
+        <v>74.099999999999994</v>
       </c>
       <c r="D35">
-        <v>15.6</v>
+        <v>89.6</v>
       </c>
       <c r="E35">
-        <v>23.5</v>
+        <v>141</v>
       </c>
       <c r="F35">
-        <v>29.5</v>
+        <v>178</v>
       </c>
       <c r="G35">
-        <v>38.799999999999997</v>
+        <v>217</v>
       </c>
       <c r="H35">
-        <v>57.2</v>
+        <v>266</v>
       </c>
       <c r="I35">
-        <v>68.8</v>
+        <v>304</v>
       </c>
       <c r="J35">
-        <v>76.3</v>
+        <v>342</v>
       </c>
       <c r="K35">
-        <v>109</v>
+        <v>394</v>
       </c>
       <c r="L35">
-        <v>111</v>
+        <v>435</v>
       </c>
       <c r="M35">
-        <v>140</v>
-      </c>
-      <c r="N35">
-        <v>173</v>
-      </c>
-      <c r="O35">
-        <v>219</v>
-      </c>
-      <c r="P35">
-        <v>257</v>
-      </c>
-      <c r="Q35">
-        <v>297</v>
-      </c>
-      <c r="R35">
-        <v>356</v>
-      </c>
-      <c r="S35">
-        <v>405</v>
-      </c>
-      <c r="T35">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B36">
         <v>5760</v>
       </c>
       <c r="C36">
-        <v>11.8</v>
+        <v>78.2</v>
       </c>
       <c r="D36">
-        <v>16</v>
+        <v>94.6</v>
       </c>
       <c r="E36">
-        <v>24.3</v>
+        <v>148</v>
       </c>
       <c r="F36">
-        <v>30.7</v>
+        <v>186</v>
       </c>
       <c r="G36">
-        <v>40.6</v>
+        <v>225</v>
       </c>
       <c r="H36">
-        <v>60</v>
+        <v>274</v>
       </c>
       <c r="I36">
-        <v>72</v>
+        <v>311</v>
       </c>
       <c r="J36">
-        <v>80</v>
+        <v>349</v>
       </c>
       <c r="K36">
-        <v>114</v>
+        <v>399</v>
       </c>
       <c r="L36">
-        <v>116</v>
+        <v>438</v>
       </c>
       <c r="M36">
-        <v>145</v>
-      </c>
-      <c r="N36">
-        <v>179</v>
-      </c>
-      <c r="O36">
-        <v>225</v>
-      </c>
-      <c r="P36">
-        <v>263</v>
-      </c>
-      <c r="Q36">
-        <v>303</v>
-      </c>
-      <c r="R36">
-        <v>364</v>
-      </c>
-      <c r="S36">
-        <v>413</v>
-      </c>
-      <c r="T36">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B37">
         <v>7200</v>
       </c>
       <c r="C37">
-        <v>11.9</v>
+        <v>80.900000000000006</v>
       </c>
       <c r="D37">
-        <v>16.3</v>
+        <v>97.9</v>
       </c>
       <c r="E37">
-        <v>25</v>
+        <v>153</v>
       </c>
       <c r="F37">
-        <v>31.7</v>
+        <v>191</v>
       </c>
       <c r="G37">
-        <v>42.1</v>
+        <v>231</v>
       </c>
       <c r="H37">
-        <v>62.5</v>
+        <v>279</v>
       </c>
       <c r="I37">
-        <v>75</v>
+        <v>316</v>
       </c>
       <c r="J37">
-        <v>83.3</v>
+        <v>353</v>
       </c>
       <c r="K37">
-        <v>118</v>
+        <v>403</v>
       </c>
       <c r="L37">
-        <v>120</v>
+        <v>440</v>
       </c>
       <c r="M37">
-        <v>150</v>
-      </c>
-      <c r="N37">
-        <v>184</v>
-      </c>
-      <c r="O37">
-        <v>230</v>
-      </c>
-      <c r="P37">
-        <v>267</v>
-      </c>
-      <c r="Q37">
-        <v>306</v>
-      </c>
-      <c r="R37">
-        <v>368</v>
-      </c>
-      <c r="S37">
-        <v>418</v>
-      </c>
-      <c r="T37">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B38">
         <v>8640</v>
       </c>
       <c r="C38">
-        <v>12</v>
+        <v>82.9</v>
       </c>
       <c r="D38">
-        <v>16.399999999999999</v>
+        <v>100</v>
       </c>
       <c r="E38">
-        <v>25.5</v>
+        <v>156</v>
       </c>
       <c r="F38">
-        <v>32.700000000000003</v>
+        <v>195</v>
       </c>
       <c r="G38">
-        <v>43.7</v>
+        <v>234</v>
       </c>
       <c r="H38">
-        <v>65.099999999999994</v>
+        <v>283</v>
       </c>
       <c r="I38">
-        <v>78</v>
+        <v>319</v>
       </c>
       <c r="J38">
-        <v>86.5</v>
+        <v>356</v>
       </c>
       <c r="K38">
-        <v>122</v>
+        <v>406</v>
       </c>
       <c r="L38">
-        <v>124</v>
+        <v>444</v>
       </c>
       <c r="M38">
-        <v>154</v>
-      </c>
-      <c r="N38">
-        <v>188</v>
-      </c>
-      <c r="O38">
-        <v>234</v>
-      </c>
-      <c r="P38">
-        <v>271</v>
-      </c>
-      <c r="Q38">
-        <v>309</v>
-      </c>
-      <c r="R38">
-        <v>372</v>
-      </c>
-      <c r="S38">
-        <v>422</v>
-      </c>
-      <c r="T38">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B39">
         <v>10080</v>
       </c>
       <c r="C39">
-        <v>12</v>
+        <v>84.3</v>
       </c>
       <c r="D39">
-        <v>16.399999999999999</v>
+        <v>102</v>
       </c>
       <c r="E39">
-        <v>26</v>
+        <v>158</v>
       </c>
       <c r="F39">
-        <v>33.6</v>
+        <v>198</v>
       </c>
       <c r="G39">
-        <v>45.2</v>
+        <v>237</v>
       </c>
       <c r="H39">
-        <v>67.7</v>
+        <v>286</v>
       </c>
       <c r="I39">
-        <v>81</v>
+        <v>323</v>
       </c>
       <c r="J39">
-        <v>89.9</v>
+        <v>359</v>
       </c>
       <c r="K39">
-        <v>126</v>
+        <v>411</v>
       </c>
       <c r="L39">
-        <v>128</v>
+        <v>449</v>
       </c>
       <c r="M39">
-        <v>159</v>
-      </c>
-      <c r="N39">
-        <v>193</v>
-      </c>
-      <c r="O39">
-        <v>239</v>
-      </c>
-      <c r="P39">
-        <v>275</v>
-      </c>
-      <c r="Q39">
-        <v>312</v>
-      </c>
-      <c r="R39">
-        <v>375</v>
-      </c>
-      <c r="S39">
-        <v>426</v>
-      </c>
-      <c r="T39">
-        <v>480</v>
+        <v>498</v>
       </c>
     </row>
   </sheetData>
@@ -3064,84 +2413,63 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFD455F-8B0B-4EE8-A131-54EC52F3D2BE}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:Y37"/>
+  <dimension ref="A1:Z37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B1">
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" t="str" cm="1">
-        <f t="array" ref="H1:Y1">_xlfn.LET(
+        <v>49</v>
+      </c>
+      <c r="H1" cm="1">
+        <f t="array" ref="H1:R1">_xlfn.LET(
 _xlpm.data,raw_IFD!C10:AZ10,
 _xlpm.filtered,_xlfn._xlws.FILTER((_xlpm.data),_xlpm.data&lt;&gt;0),
 _xlpm.filtered
 )</f>
-        <v>12EY</v>
-      </c>
-      <c r="I1" t="str">
-        <v>6EY</v>
-      </c>
-      <c r="J1" t="str">
-        <v>4EY</v>
-      </c>
-      <c r="K1" t="str">
-        <v>3EY</v>
-      </c>
-      <c r="L1" t="str">
-        <v>2EY</v>
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="I1">
+        <v>0.5</v>
+      </c>
+      <c r="J1">
+        <v>0.2</v>
+      </c>
+      <c r="K1">
+        <v>0.1</v>
+      </c>
+      <c r="L1">
+        <v>0.05</v>
       </c>
       <c r="M1">
-        <v>0.63200000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="N1">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="O1" t="str">
-        <v>0.5EY</v>
-      </c>
-      <c r="P1">
-        <v>0.2</v>
+        <v>1 in 200</v>
+      </c>
+      <c r="P1" t="str">
+        <v>1 in 500</v>
       </c>
       <c r="Q1" t="str">
-        <v>0.2EY</v>
-      </c>
-      <c r="R1">
-        <v>0.1</v>
-      </c>
-      <c r="S1">
-        <v>0.05</v>
-      </c>
-      <c r="T1">
-        <v>0.02</v>
-      </c>
-      <c r="U1">
-        <v>0.01</v>
-      </c>
-      <c r="V1" t="str">
-        <v>1 in 200</v>
-      </c>
-      <c r="W1" t="str">
-        <v>1 in 500</v>
-      </c>
-      <c r="X1" t="str">
         <v>1 in 1000</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="R1" t="str">
         <v>1 in 2000</v>
       </c>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="str">
         <f>raw_IFD!C7</f>
         <v>22.5875 (S)</v>
@@ -3151,65 +2479,44 @@
         <v>22.5875</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H2" s="2" t="str" cm="1">
-        <f t="array" ref="H2:Y2">_xlfn.XLOOKUP(_xlfn.ANCHORARRAY(H1),raw_IFD!10:10,raw_IFD!10:10,NA(),0)</f>
-        <v>12EY</v>
-      </c>
-      <c r="I2" s="2" t="str">
-        <v>6EY</v>
-      </c>
-      <c r="J2" s="2" t="str">
-        <v>4EY</v>
-      </c>
-      <c r="K2" s="2" t="str">
-        <v>3EY</v>
-      </c>
-      <c r="L2" s="2" t="str">
-        <v>2EY</v>
+        <v>50</v>
+      </c>
+      <c r="H2" s="2" cm="1">
+        <f t="array" ref="H2:R2">_xlfn.XLOOKUP(_xlfn.ANCHORARRAY(H1),raw_IFD!10:10,raw_IFD!10:10,NA(),0)</f>
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.05</v>
       </c>
       <c r="M2" s="2">
-        <v>0.63200000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="N2" s="2">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="O2" s="2" t="str">
-        <v>0.5EY</v>
-      </c>
-      <c r="P2" s="2">
-        <v>0.2</v>
+        <v>1 in 200</v>
+      </c>
+      <c r="P2" s="2" t="str">
+        <v>1 in 500</v>
       </c>
       <c r="Q2" s="2" t="str">
-        <v>0.2EY</v>
-      </c>
-      <c r="R2" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="S2" s="2">
-        <v>0.05</v>
-      </c>
-      <c r="T2" s="2">
-        <v>0.02</v>
-      </c>
-      <c r="U2" s="2">
-        <v>0.01</v>
-      </c>
-      <c r="V2" s="2" t="str">
-        <v>1 in 200</v>
-      </c>
-      <c r="W2" s="2" t="str">
-        <v>1 in 500</v>
-      </c>
-      <c r="X2" s="2" t="str">
         <v>1 in 1000</v>
       </c>
-      <c r="Y2" s="2" t="str">
+      <c r="R2" s="2" t="str">
         <v>1 in 2000</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>raw_IFD!E7</f>
         <v>117.0125 (E)</v>
@@ -3219,10 +2526,7 @@
         <v>117.0125</v>
       </c>
       <c r="G3" t="s">
-        <v>53</v>
-      </c>
-      <c r="M3">
-        <v>0.63200000000000001</v>
+        <v>45</v>
       </c>
       <c r="N3">
         <v>0.5</v>
@@ -3242,131 +2546,143 @@
       <c r="U3">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="V3" t="s">
+        <v>11</v>
+      </c>
+      <c r="W3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G4" s="2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="H4" s="2" cm="1">
-        <f t="array" ref="H4:N4">_xlfn.LET(
+        <f t="array" ref="H4:O4">_xlfn.LET(
     _xlpm.source,_xlfn.ANCHORARRAY( H1),
     _xlpm.filterCriteria, H3:AZ3,
     _xlpm.filteredResults, _xlfn._xlws.FILTER(_xlpm.source, COUNTIF(_xlpm.filterCriteria, _xlpm.source) &gt; 0),
     _xlpm.filteredResults
 )</f>
-        <v>0.63200000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="N4" s="2" t="str">
+        <v>1 in 200</v>
+      </c>
+      <c r="O4" s="2" t="str">
+        <v>1 in 500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="2" cm="1">
+        <f t="array" ref="H5:O5">_xlfn.XLOOKUP(_xlfn.ANCHORARRAY(H4),_xlfn.ANCHORARRAY(H1),_xlfn.ANCHORARRAY(H2),NA(),0)</f>
         <v>0.5</v>
       </c>
-      <c r="J4" s="2">
+      <c r="I5" s="2">
         <v>0.2</v>
       </c>
-      <c r="K4" s="2">
+      <c r="J5" s="2">
         <v>0.1</v>
       </c>
-      <c r="L4" s="2">
+      <c r="K5" s="2">
         <v>0.05</v>
       </c>
-      <c r="M4" s="2">
+      <c r="L5" s="2">
         <v>0.02</v>
       </c>
-      <c r="N4" s="2">
+      <c r="M5" s="2">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="G5" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="2" cm="1">
-        <f t="array" ref="H5:N5">_xlfn.XLOOKUP(_xlfn.ANCHORARRAY(H4),_xlfn.ANCHORARRAY(H1),_xlfn.ANCHORARRAY(H2),NA(),0)</f>
-        <v>0.63200000000000001</v>
-      </c>
-      <c r="I5" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="K5" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="L5" s="2">
-        <v>0.05</v>
-      </c>
-      <c r="M5" s="2">
-        <v>0.02</v>
-      </c>
-      <c r="N5" s="2">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="N5" s="2" t="str">
+        <v>1 in 200</v>
+      </c>
+      <c r="O5" s="2" t="str">
+        <v>1 in 500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="G7" s="2" t="str">
-        <f>_xlfn.CONCAT("IFD data for ",B2, "°S, ", B3,"°E")</f>
-        <v>IFD data for 22.5875°S, 117.0125°E</v>
+        <f>_xlfn.CONCAT("IFD data for ",B2, "°S, ", B3,"°E (rainfall event depth, mm)")</f>
+        <v>IFD data for 22.5875°S, 117.0125°E (rainfall event depth, mm)</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q7" s="7" t="str">
+        <v>54</v>
+      </c>
+      <c r="R7" s="7" t="str">
         <f>G7</f>
-        <v>IFD data for 22.5875°S, 117.0125°E</v>
-      </c>
-      <c r="X7" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>IFD data for 22.5875°S, 117.0125°E (rainfall event depth, mm)</v>
+      </c>
+      <c r="Y7" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H8" s="4" cm="1">
-        <f t="array" ref="H8:N8">_xlfn.ANCHORARRAY(H5)</f>
-        <v>0.63200000000000001</v>
+        <f t="array" ref="H8:O8">_xlfn.ANCHORARRAY(H5)</f>
+        <v>0.5</v>
       </c>
       <c r="I8" s="5">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="J8" s="5">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K8" s="5">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="L8" s="5">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="M8" s="5">
-        <v>0.02</v>
-      </c>
-      <c r="N8" s="5">
         <v>0.01</v>
       </c>
-      <c r="Q8" s="2" t="s">
+      <c r="N8" s="5" t="str">
+        <v>1 in 200</v>
+      </c>
+      <c r="O8" s="2" t="str">
+        <v>1 in 500</v>
+      </c>
+      <c r="R8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="R8" s="4" cm="1">
-        <f t="array" ref="R8:X8">_xlfn.ANCHORARRAY(H8)</f>
-        <v>0.63200000000000001</v>
-      </c>
-      <c r="S8" s="5">
+      <c r="S8" s="4" cm="1">
+        <f t="array" ref="S8:Z8">_xlfn.ANCHORARRAY(H8)</f>
         <v>0.5</v>
       </c>
       <c r="T8" s="5">
@@ -3384,8 +2700,14 @@
       <c r="X8" s="5">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y8" s="5" t="str">
+        <v>1 in 200</v>
+      </c>
+      <c r="Z8" s="2" t="str">
+        <v>1 in 500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" cm="1">
         <f t="array" ref="A9:A37">_xlfn.LET(
     _xlpm.data, raw_IFD!B11:B50,
@@ -3416,7 +2738,7 @@
         <v>1 hour</v>
       </c>
       <c r="H9" s="3" t="str" cm="1">
-        <f t="array" ref="H9:N20">_xlfn.LET(
+        <f t="array" ref="H9:O20">_xlfn.LET(
     _xlpm.columnHeader,_xlfn.ANCHORARRAY( H8),
     _xlpm.rowLabel,_xlfn.ANCHORARRAY( G9),
     _xlpm.dataRange, raw_IFD!C11:AZ200,
@@ -3433,32 +2755,35 @@
     ),
     _xlpm.formattedValue
 )</f>
-        <v>22.1</v>
+        <v>26.4</v>
       </c>
       <c r="I9" s="3" t="str">
-        <v>25.5</v>
+        <v>37.9</v>
       </c>
       <c r="J9" s="3" t="str">
-        <v>36.2</v>
+        <v>45.8</v>
       </c>
       <c r="K9" s="3" t="str">
-        <v>43.4</v>
+        <v>53.7</v>
       </c>
       <c r="L9" s="3" t="str">
-        <v>50.6</v>
+        <v>64.1</v>
       </c>
       <c r="M9" s="3" t="str">
-        <v>60.2</v>
+        <v>72.2</v>
       </c>
       <c r="N9" s="3" t="str">
-        <v>67.6</v>
-      </c>
-      <c r="Q9" t="str" cm="1">
-        <f t="array" ref="Q9:Q20">_xlfn.ANCHORARRAY(G9)</f>
+        <v>82.3</v>
+      </c>
+      <c r="O9" t="str">
+        <v>96.8</v>
+      </c>
+      <c r="R9" t="str" cm="1">
+        <f t="array" ref="R9:R20">_xlfn.ANCHORARRAY(G9)</f>
         <v>1 hour</v>
       </c>
-      <c r="R9" s="3" t="str" cm="1">
-        <f t="array" ref="R9:X20">_xlfn.LET(
+      <c r="S9" s="3" t="str" cm="1">
+        <f t="array" ref="S9:Z20">_xlfn.LET(
     _xlpm.columnHeader,_xlfn.ANCHORARRAY( H8),
     _xlpm.rowLabel,_xlfn.ANCHORARRAY( G9),
     _xlpm.dataRange, raw_IFD!C11:AZ200,
@@ -3479,28 +2804,31 @@
     ),
     _xlpm.formattedValue
 )</f>
-        <v>22.1</v>
-      </c>
-      <c r="S9" s="3" t="str">
-        <v>25.5</v>
+        <v>26.4</v>
       </c>
       <c r="T9" s="3" t="str">
-        <v>36.2</v>
+        <v>37.9</v>
       </c>
       <c r="U9" s="3" t="str">
-        <v>43.4</v>
+        <v>45.8</v>
       </c>
       <c r="V9" s="3" t="str">
-        <v>50.6</v>
+        <v>53.7</v>
       </c>
       <c r="W9" s="3" t="str">
-        <v>60.2</v>
+        <v>64.1</v>
       </c>
       <c r="X9" s="3" t="str">
-        <v>67.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+        <v>72.2</v>
+      </c>
+      <c r="Y9" s="3" t="str">
+        <v>82.3</v>
+      </c>
+      <c r="Z9" t="str">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
@@ -3517,52 +2845,58 @@
         <v>2 hour</v>
       </c>
       <c r="H10" s="3" t="str">
-        <v>27.1</v>
+        <v>32.3</v>
       </c>
       <c r="I10" s="3" t="str">
-        <v>31.3</v>
+        <v>46.9</v>
       </c>
       <c r="J10" s="3" t="str">
-        <v>44.6</v>
+        <v>57.1</v>
       </c>
       <c r="K10" s="3" t="str">
-        <v>53.8</v>
+        <v>67.2</v>
       </c>
       <c r="L10" s="3" t="str">
-        <v>62.9</v>
+        <v>80.9</v>
       </c>
       <c r="M10" s="3" t="str">
-        <v>75.1</v>
+        <v>91.7</v>
       </c>
       <c r="N10" s="3" t="str">
-        <v>84.6</v>
-      </c>
-      <c r="Q10" t="str">
+        <v>104</v>
+      </c>
+      <c r="O10" t="str">
+        <v>123</v>
+      </c>
+      <c r="R10" t="str">
         <v>2 hour</v>
       </c>
-      <c r="R10" s="3" t="str">
-        <v>27.1</v>
-      </c>
       <c r="S10" s="3" t="str">
-        <v>31.3</v>
+        <v>32.3</v>
       </c>
       <c r="T10" s="3" t="str">
-        <v>44.6</v>
+        <v>46.9</v>
       </c>
       <c r="U10" s="3" t="str">
-        <v>53.8</v>
+        <v>57.1</v>
       </c>
       <c r="V10" s="3" t="str">
-        <v>62.9</v>
+        <v>67.2</v>
       </c>
       <c r="W10" s="3" t="str">
-        <v>75.1</v>
+        <v>80.9</v>
       </c>
       <c r="X10" s="3" t="str">
-        <v>84.6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+        <v>91.7</v>
+      </c>
+      <c r="Y10" s="3" t="str">
+        <v>104</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>3</v>
       </c>
@@ -3579,52 +2913,58 @@
         <v>3 hour</v>
       </c>
       <c r="H11" s="3" t="str">
-        <v>30.0</v>
+        <v>36.2</v>
       </c>
       <c r="I11" s="3" t="str">
-        <v>34.8</v>
+        <v>53.0</v>
       </c>
       <c r="J11" s="3" t="str">
-        <v>50.2</v>
+        <v>64.9</v>
       </c>
       <c r="K11" s="3" t="str">
-        <v>60.9</v>
+        <v>76.9</v>
       </c>
       <c r="L11" s="3" t="str">
-        <v>71.5</v>
+        <v>93.4</v>
       </c>
       <c r="M11" s="3" t="str">
-        <v>85.9</v>
+        <v>106</v>
       </c>
       <c r="N11" s="3" t="str">
-        <v>97.2</v>
-      </c>
-      <c r="Q11" t="str">
+        <v>121</v>
+      </c>
+      <c r="O11" t="str">
+        <v>143</v>
+      </c>
+      <c r="R11" t="str">
         <v>3 hour</v>
       </c>
-      <c r="R11" s="3" t="str">
-        <v>30.0</v>
-      </c>
       <c r="S11" s="3" t="str">
-        <v>34.8</v>
+        <v>36.2</v>
       </c>
       <c r="T11" s="3" t="str">
-        <v>50.2</v>
+        <v>53.0</v>
       </c>
       <c r="U11" s="3" t="str">
-        <v>60.9</v>
+        <v>64.9</v>
       </c>
       <c r="V11" s="3" t="str">
-        <v>71.5</v>
+        <v>76.9</v>
       </c>
       <c r="W11" s="3" t="str">
-        <v>85.9</v>
+        <v>93.4</v>
       </c>
       <c r="X11" s="3" t="str">
-        <v>97.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+      <c r="Y11" s="3" t="str">
+        <v>121</v>
+      </c>
+      <c r="Z11" t="str">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>4</v>
       </c>
@@ -3641,52 +2981,58 @@
         <v>6 hour</v>
       </c>
       <c r="H12" s="3" t="str">
-        <v>35.5</v>
+        <v>44.1</v>
       </c>
       <c r="I12" s="3" t="str">
-        <v>41.6</v>
+        <v>66.2</v>
       </c>
       <c r="J12" s="3" t="str">
-        <v>61.4</v>
+        <v>82.2</v>
       </c>
       <c r="K12" s="3" t="str">
-        <v>75.5</v>
+        <v>98.7</v>
       </c>
       <c r="L12" s="3" t="str">
-        <v>89.9</v>
+        <v>122</v>
       </c>
       <c r="M12" s="3" t="str">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="N12" s="3" t="str">
-        <v>125</v>
-      </c>
-      <c r="Q12" t="str">
+        <v>160</v>
+      </c>
+      <c r="O12" t="str">
+        <v>189</v>
+      </c>
+      <c r="R12" t="str">
         <v>6 hour</v>
       </c>
-      <c r="R12" s="3" t="str">
-        <v>35.5</v>
-      </c>
       <c r="S12" s="3" t="str">
-        <v>41.6</v>
+        <v>44.1</v>
       </c>
       <c r="T12" s="3" t="str">
-        <v>61.4</v>
+        <v>66.2</v>
       </c>
       <c r="U12" s="3" t="str">
-        <v>75.5</v>
+        <v>82.2</v>
       </c>
       <c r="V12" s="3" t="str">
-        <v>89.9</v>
+        <v>98.7</v>
       </c>
       <c r="W12" s="3" t="str">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="X12" s="3" t="str">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+      <c r="Y12" s="3" t="str">
+        <v>160</v>
+      </c>
+      <c r="Z12" t="str">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5</v>
       </c>
@@ -3703,52 +3049,58 @@
         <v>9 hour</v>
       </c>
       <c r="H13" s="3" t="str">
-        <v>38.9</v>
+        <v>49.8</v>
       </c>
       <c r="I13" s="3" t="str">
-        <v>45.9</v>
+        <v>76.0</v>
       </c>
       <c r="J13" s="3" t="str">
-        <v>69.0</v>
+        <v>95.2</v>
       </c>
       <c r="K13" s="3" t="str">
-        <v>85.8</v>
+        <v>115</v>
       </c>
       <c r="L13" s="3" t="str">
-        <v>103</v>
+        <v>143</v>
       </c>
       <c r="M13" s="3" t="str">
-        <v>127</v>
+        <v>166</v>
       </c>
       <c r="N13" s="3" t="str">
-        <v>147</v>
-      </c>
-      <c r="Q13" t="str">
+        <v>189</v>
+      </c>
+      <c r="O13" t="str">
+        <v>224</v>
+      </c>
+      <c r="R13" t="str">
         <v>9 hour</v>
       </c>
-      <c r="R13" s="3" t="str">
-        <v>38.9</v>
-      </c>
       <c r="S13" s="3" t="str">
-        <v>45.9</v>
+        <v>49.8</v>
       </c>
       <c r="T13" s="3" t="str">
-        <v>69.0</v>
+        <v>76.0</v>
       </c>
       <c r="U13" s="3" t="str">
-        <v>85.8</v>
+        <v>95.2</v>
       </c>
       <c r="V13" s="3" t="str">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="W13" s="3" t="str">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="X13" s="3" t="str">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+      <c r="Y13" s="3" t="str">
+        <v>189</v>
+      </c>
+      <c r="Z13" t="str">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -3765,52 +3117,58 @@
         <v>12 hour</v>
       </c>
       <c r="H14" s="3" t="str">
-        <v>41.5</v>
+        <v>54.4</v>
       </c>
       <c r="I14" s="3" t="str">
-        <v>49.1</v>
+        <v>83.9</v>
       </c>
       <c r="J14" s="3" t="str">
-        <v>74.8</v>
+        <v>106</v>
       </c>
       <c r="K14" s="3" t="str">
-        <v>93.7</v>
+        <v>128</v>
       </c>
       <c r="L14" s="3" t="str">
-        <v>113</v>
+        <v>160</v>
       </c>
       <c r="M14" s="3" t="str">
-        <v>141</v>
+        <v>186</v>
       </c>
       <c r="N14" s="3" t="str">
-        <v>164</v>
-      </c>
-      <c r="Q14" t="str">
+        <v>213</v>
+      </c>
+      <c r="O14" t="str">
+        <v>252</v>
+      </c>
+      <c r="R14" t="str">
         <v>12 hour</v>
       </c>
-      <c r="R14" s="3" t="str">
-        <v>41.5</v>
-      </c>
       <c r="S14" s="3" t="str">
-        <v>49.1</v>
+        <v>54.4</v>
       </c>
       <c r="T14" s="3" t="str">
-        <v>74.8</v>
+        <v>83.9</v>
       </c>
       <c r="U14" s="3" t="str">
-        <v>93.7</v>
+        <v>106</v>
       </c>
       <c r="V14" s="3" t="str">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="W14" s="3" t="str">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="X14" s="3" t="str">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+      <c r="Y14" s="3" t="str">
+        <v>213</v>
+      </c>
+      <c r="Z14" t="str">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>15</v>
       </c>
@@ -3827,52 +3185,58 @@
         <v>18 hour</v>
       </c>
       <c r="H15" s="3" t="str">
-        <v>45.1</v>
+        <v>61.7</v>
       </c>
       <c r="I15" s="3" t="str">
-        <v>53.8</v>
+        <v>96.4</v>
       </c>
       <c r="J15" s="3" t="str">
-        <v>83.2</v>
+        <v>122</v>
       </c>
       <c r="K15" s="3" t="str">
-        <v>105</v>
+        <v>149</v>
       </c>
       <c r="L15" s="3" t="str">
-        <v>129</v>
+        <v>187</v>
       </c>
       <c r="M15" s="3" t="str">
-        <v>162</v>
+        <v>218</v>
       </c>
       <c r="N15" s="3" t="str">
-        <v>189</v>
-      </c>
-      <c r="Q15" t="str">
+        <v>248</v>
+      </c>
+      <c r="O15" t="str">
+        <v>293</v>
+      </c>
+      <c r="R15" t="str">
         <v>18 hour</v>
       </c>
-      <c r="R15" s="3" t="str">
-        <v>45.1</v>
-      </c>
       <c r="S15" s="3" t="str">
-        <v>53.8</v>
+        <v>61.7</v>
       </c>
       <c r="T15" s="3" t="str">
-        <v>83.2</v>
+        <v>96.4</v>
       </c>
       <c r="U15" s="3" t="str">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="V15" s="3" t="str">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="W15" s="3" t="str">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="X15" s="3" t="str">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="Y15" s="3" t="str">
+        <v>248</v>
+      </c>
+      <c r="Z15" t="str">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>20</v>
       </c>
@@ -3889,52 +3253,58 @@
         <v>24 hour</v>
       </c>
       <c r="H16" s="3" t="str">
-        <v>47.7</v>
+        <v>67.4</v>
       </c>
       <c r="I16" s="3" t="str">
-        <v>57.0</v>
+        <v>106</v>
       </c>
       <c r="J16" s="3" t="str">
-        <v>89.2</v>
+        <v>135</v>
       </c>
       <c r="K16" s="3" t="str">
-        <v>114</v>
+        <v>165</v>
       </c>
       <c r="L16" s="3" t="str">
-        <v>140</v>
+        <v>206</v>
       </c>
       <c r="M16" s="3" t="str">
-        <v>176</v>
+        <v>240</v>
       </c>
       <c r="N16" s="3" t="str">
-        <v>207</v>
-      </c>
-      <c r="Q16" t="str">
+        <v>274</v>
+      </c>
+      <c r="O16" t="str">
+        <v>323</v>
+      </c>
+      <c r="R16" t="str">
         <v>24 hour</v>
       </c>
-      <c r="R16" s="3" t="str">
-        <v>47.7</v>
-      </c>
       <c r="S16" s="3" t="str">
-        <v>57.0</v>
+        <v>67.4</v>
       </c>
       <c r="T16" s="3" t="str">
-        <v>89.2</v>
+        <v>106</v>
       </c>
       <c r="U16" s="3" t="str">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="V16" s="3" t="str">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="W16" s="3" t="str">
-        <v>176</v>
+        <v>206</v>
       </c>
       <c r="X16" s="3" t="str">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+      <c r="Y16" s="3" t="str">
+        <v>274</v>
+      </c>
+      <c r="Z16" t="str">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>25</v>
       </c>
@@ -3951,52 +3321,58 @@
         <v>30 hour</v>
       </c>
       <c r="H17" s="3" t="str">
-        <v>49.6</v>
+        <v>72.0</v>
       </c>
       <c r="I17" s="3" t="str">
-        <v>59.5</v>
+        <v>114</v>
       </c>
       <c r="J17" s="3" t="str">
-        <v>93.7</v>
+        <v>144</v>
       </c>
       <c r="K17" s="3" t="str">
-        <v>120</v>
+        <v>177</v>
       </c>
       <c r="L17" s="3" t="str">
-        <v>148</v>
+        <v>221</v>
       </c>
       <c r="M17" s="3" t="str">
-        <v>187</v>
+        <v>257</v>
       </c>
       <c r="N17" s="3" t="str">
-        <v>220</v>
-      </c>
-      <c r="Q17" t="str">
+        <v>294</v>
+      </c>
+      <c r="O17" t="str">
+        <v>347</v>
+      </c>
+      <c r="R17" t="str">
         <v>30 hour</v>
       </c>
-      <c r="R17" s="3" t="str">
-        <v>49.6</v>
-      </c>
       <c r="S17" s="3" t="str">
-        <v>59.5</v>
+        <v>72.0</v>
       </c>
       <c r="T17" s="3" t="str">
-        <v>93.7</v>
+        <v>114</v>
       </c>
       <c r="U17" s="3" t="str">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="V17" s="3" t="str">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="W17" s="3" t="str">
-        <v>187</v>
+        <v>221</v>
       </c>
       <c r="X17" s="3" t="str">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="Y17" s="3" t="str">
+        <v>294</v>
+      </c>
+      <c r="Z17" t="str">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>30</v>
       </c>
@@ -4013,52 +3389,58 @@
         <v>36 hour</v>
       </c>
       <c r="H18" s="3" t="str">
-        <v>51.2</v>
+        <v>75.8</v>
       </c>
       <c r="I18" s="3" t="str">
-        <v>61.5</v>
+        <v>120</v>
       </c>
       <c r="J18" s="3" t="str">
-        <v>97.2</v>
+        <v>152</v>
       </c>
       <c r="K18" s="3" t="str">
-        <v>124</v>
+        <v>186</v>
       </c>
       <c r="L18" s="3" t="str">
-        <v>154</v>
+        <v>232</v>
       </c>
       <c r="M18" s="3" t="str">
-        <v>195</v>
+        <v>269</v>
       </c>
       <c r="N18" s="3" t="str">
-        <v>230</v>
-      </c>
-      <c r="Q18" t="str">
+        <v>308</v>
+      </c>
+      <c r="O18" t="str">
+        <v>363</v>
+      </c>
+      <c r="R18" t="str">
         <v>36 hour</v>
       </c>
-      <c r="R18" s="3" t="str">
-        <v>51.2</v>
-      </c>
       <c r="S18" s="3" t="str">
-        <v>61.5</v>
+        <v>75.8</v>
       </c>
       <c r="T18" s="3" t="str">
-        <v>97.2</v>
+        <v>120</v>
       </c>
       <c r="U18" s="3" t="str">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="V18" s="3" t="str">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="W18" s="3" t="str">
-        <v>195</v>
+        <v>232</v>
       </c>
       <c r="X18" s="3" t="str">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+      <c r="Y18" s="3" t="str">
+        <v>308</v>
+      </c>
+      <c r="Z18" t="str">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>45</v>
       </c>
@@ -4075,52 +3457,58 @@
         <v>48 hour</v>
       </c>
       <c r="H19" s="3" t="str">
-        <v>53.7</v>
+        <v>81.7</v>
       </c>
       <c r="I19" s="3" t="str">
-        <v>64.5</v>
+        <v>129</v>
       </c>
       <c r="J19" s="3" t="str">
-        <v>102</v>
+        <v>164</v>
       </c>
       <c r="K19" s="3" t="str">
-        <v>131</v>
+        <v>200</v>
       </c>
       <c r="L19" s="3" t="str">
-        <v>163</v>
+        <v>248</v>
       </c>
       <c r="M19" s="3" t="str">
-        <v>207</v>
+        <v>286</v>
       </c>
       <c r="N19" s="3" t="str">
-        <v>243</v>
-      </c>
-      <c r="Q19" t="str">
+        <v>326</v>
+      </c>
+      <c r="O19" t="str">
+        <v>381</v>
+      </c>
+      <c r="R19" t="str">
         <v>48 hour</v>
       </c>
-      <c r="R19" s="3" t="str">
-        <v>53.7</v>
-      </c>
       <c r="S19" s="3" t="str">
-        <v>64.5</v>
+        <v>81.7</v>
       </c>
       <c r="T19" s="3" t="str">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="U19" s="3" t="str">
-        <v>131</v>
+        <v>164</v>
       </c>
       <c r="V19" s="3" t="str">
-        <v>163</v>
+        <v>200</v>
       </c>
       <c r="W19" s="3" t="str">
-        <v>207</v>
+        <v>248</v>
       </c>
       <c r="X19" s="3" t="str">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+      <c r="Y19" s="3" t="str">
+        <v>326</v>
+      </c>
+      <c r="Z19" t="str">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>60</v>
       </c>
@@ -4140,52 +3528,58 @@
         <v>72 hour</v>
       </c>
       <c r="H20" s="3" t="str">
-        <v>57.2</v>
+        <v>89.6</v>
       </c>
       <c r="I20" s="3" t="str">
-        <v>68.8</v>
+        <v>141</v>
       </c>
       <c r="J20" s="3" t="str">
-        <v>109</v>
+        <v>178</v>
       </c>
       <c r="K20" s="3" t="str">
-        <v>140</v>
+        <v>217</v>
       </c>
       <c r="L20" s="3" t="str">
-        <v>173</v>
+        <v>266</v>
       </c>
       <c r="M20" s="3" t="str">
-        <v>219</v>
+        <v>304</v>
       </c>
       <c r="N20" s="3" t="str">
-        <v>257</v>
-      </c>
-      <c r="Q20" t="str">
+        <v>342</v>
+      </c>
+      <c r="O20" t="str">
+        <v>394</v>
+      </c>
+      <c r="R20" t="str">
         <v>72 hour</v>
       </c>
-      <c r="R20" s="3" t="str">
-        <v>57.2</v>
-      </c>
       <c r="S20" s="3" t="str">
-        <v>68.8</v>
+        <v>89.6</v>
       </c>
       <c r="T20" s="3" t="str">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="U20" s="3" t="str">
-        <v>140</v>
+        <v>178</v>
       </c>
       <c r="V20" s="3" t="str">
-        <v>173</v>
+        <v>217</v>
       </c>
       <c r="W20" s="3" t="str">
-        <v>219</v>
+        <v>266</v>
       </c>
       <c r="X20" s="3" t="str">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+        <v>304</v>
+      </c>
+      <c r="Y20" s="3" t="str">
+        <v>342</v>
+      </c>
+      <c r="Z20" t="str">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>90</v>
       </c>
@@ -4200,7 +3594,7 @@
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>120</v>
       </c>
@@ -4218,7 +3612,7 @@
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>180</v>
       </c>
@@ -4236,7 +3630,7 @@
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>270</v>
       </c>
@@ -4251,7 +3645,7 @@
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>360</v>
       </c>
@@ -4269,7 +3663,7 @@
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>540</v>
       </c>
@@ -4287,7 +3681,7 @@
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>720</v>
       </c>
@@ -4305,7 +3699,7 @@
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1080</v>
       </c>
@@ -4316,7 +3710,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1440</v>
       </c>
@@ -4327,7 +3721,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1800</v>
       </c>
@@ -4338,7 +3732,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2160</v>
       </c>
@@ -4349,7 +3743,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2880</v>
       </c>

</xml_diff>